<commit_message>
Update data package at: 2026-09-23T14:34:16Z
</commit_message>
<xml_diff>
--- a/data-raw/desc_base_legal_demonstrativos.xlsx
+++ b/data-raw/desc_base_legal_demonstrativos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cecad365.sharepoint.com/sites/Splor/Documentos Compartilhados/General/@dcppn/DCPPN 2026/PPAG e LOA 2026/material de apoio/material de apoio - gerar volumes/2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cecad365.sharepoint.com/sites/Splor/Documentos Compartilhados/General/@dcppn/00- DCPPN 2027/PPAG e LOA 2027/Dados para Volumes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="416" documentId="11_A3DD8646BA7476893AAB1FDD9F017BEA3498940F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AABACC1-D64D-48C7-8AD2-BF49F9BB0DE6}"/>
+  <xr:revisionPtr revIDLastSave="456" documentId="11_A3DD8646BA7476893AAB1FDD9F017BEA3498940F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D198958F-0B4B-44B4-A2D2-2146EB82D29B}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="base_legal" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <externalReference r:id="rId3"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">base_legal!$B$1:$C$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">base_legal!$B$1:$C$30</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="156">
   <si>
     <t>cod</t>
   </si>
@@ -452,6 +452,66 @@
   </si>
   <si>
     <t>PEdro</t>
+  </si>
+  <si>
+    <t>(Art. 7º, Inciso XXII da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 7º, Inciso XXIII da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 7º, Inciso II da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 7º, Inciso XV da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 212 da Constituição Federal, Art. 201 da Constituição Estadual e Art. 7º, Inciso III da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 158,  §1º da Constituição Estadual e Art. 7º, Inciso IV da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 198 da Constituição Federal e Art. 7°, Inciso V da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 212 da Constituição Estadual e Art. 7°, Inciso VI da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 19 da Lei Complementar 101/2000 - LRF e Art. 7°, Inciso VIII da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 7º, Inciso XIII da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 7º, Inciso XVIII da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 7º, Inciso X da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 7º, Inciso XI da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 7º, Inciso XXV da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 31 da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 7º, Inciso XVII da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 32 da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 7º, Inciso XX da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>(Art. 7º, Inciso I da Lei 26.041/2026 - LDO)</t>
+  </si>
+  <si>
+    <t>T1_DEMONSTRATIVO_CONSOLIDADO_ORCAMENTO_FISCAL</t>
   </si>
 </sst>
 </file>
@@ -632,6 +692,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Controle de conferencia LOA"/>
@@ -1524,16 +1585,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="105" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="197.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="116" customWidth="1"/>
+    <col min="1" max="1" width="71.88671875" customWidth="1"/>
+    <col min="2" max="2" width="86.44140625" customWidth="1"/>
+    <col min="3" max="3" width="49.5546875" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1544,323 +1605,334 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="C5" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="C6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>16</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>19</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>20</v>
       </c>
-      <c r="C8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="C9" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>21</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>22</v>
       </c>
-      <c r="C9" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="C10" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>23</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>24</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C11" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>26</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>27</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>28</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>29</v>
-      </c>
-      <c r="C12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" t="s">
-        <v>31</v>
       </c>
       <c r="C13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>32</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>33</v>
       </c>
-      <c r="C14" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="C15" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>34</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>35</v>
       </c>
-      <c r="C15" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="C16" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>36</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>37</v>
       </c>
-      <c r="C16" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="C17" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>38</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>39</v>
       </c>
-      <c r="C17" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="C18" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>40</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B19" t="s">
         <v>41</v>
       </c>
-      <c r="C18" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="C19" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>42</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B20" t="s">
         <v>43</v>
       </c>
-      <c r="C19" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="C20" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>44</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
         <v>45</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C21" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>46</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B22" t="s">
         <v>47</v>
       </c>
-      <c r="C21" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="C22" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>48</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" t="s">
         <v>49</v>
       </c>
-      <c r="C22" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="C23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>50</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>51</v>
       </c>
-      <c r="C23" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="C24" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>52</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B25" t="s">
         <v>53</v>
       </c>
-      <c r="C24" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="C25" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>54</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B26" t="s">
         <v>55</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C26" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
         <v>57</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>58</v>
       </c>
-      <c r="C26" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="C27" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>59</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B28" t="s">
         <v>60</v>
       </c>
-      <c r="C27" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="C28" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>61</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>62</v>
       </c>
-      <c r="C28" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="C29" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
         <v>63</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B30" t="s">
         <v>64</v>
       </c>
-      <c r="C29" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="C30" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
         <v>65</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>66</v>
       </c>
-      <c r="C30" t="s">
-        <v>105</v>
+      <c r="C31" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -1872,17 +1944,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9730DD9-C36A-40E7-998B-E00A0695F1C5}">
   <dimension ref="A1:K50"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="65.5703125" customWidth="1"/>
-    <col min="2" max="2" width="33.140625" customWidth="1"/>
-    <col min="3" max="8" width="9.140625" style="6"/>
-    <col min="9" max="9" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="65.5546875" customWidth="1"/>
+    <col min="2" max="2" width="33.109375" customWidth="1"/>
+    <col min="3" max="8" width="9.109375" style="6"/>
+    <col min="9" max="9" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>67</v>
       </c>
@@ -1917,7 +1989,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>75</v>
       </c>
@@ -1932,7 +2004,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1947,7 +2019,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1962,7 +2034,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
@@ -1976,7 +2048,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
@@ -1990,7 +2062,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>14</v>
       </c>
@@ -2005,7 +2077,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
@@ -2020,7 +2092,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
@@ -2035,7 +2107,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2050,7 +2122,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>82</v>
       </c>
@@ -2065,7 +2137,7 @@
         <v>sofia</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -2080,7 +2152,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>24</v>
       </c>
@@ -2095,7 +2167,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>27</v>
       </c>
@@ -2110,7 +2182,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="24" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>29</v>
       </c>
@@ -2124,7 +2196,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="24" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>31</v>
       </c>
@@ -2138,7 +2210,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>33</v>
       </c>
@@ -2153,7 +2225,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>35</v>
       </c>
@@ -2168,7 +2240,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>37</v>
       </c>
@@ -2183,7 +2255,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>39</v>
       </c>
@@ -2198,7 +2270,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>41</v>
       </c>
@@ -2213,7 +2285,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
         <v>90</v>
       </c>
@@ -2228,7 +2300,7 @@
         <v>sofia</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="36" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="36" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
         <v>92</v>
       </c>
@@ -2243,7 +2315,7 @@
         <v>sofia</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
         <v>43</v>
       </c>
@@ -2258,7 +2330,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
         <v>95</v>
       </c>
@@ -2273,7 +2345,7 @@
         <v>sofia</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>45</v>
       </c>
@@ -2288,7 +2360,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>47</v>
       </c>
@@ -2304,7 +2376,7 @@
         <v>carolina</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>49</v>
       </c>
@@ -2319,7 +2391,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>51</v>
       </c>
@@ -2334,7 +2406,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>53</v>
       </c>
@@ -2349,7 +2421,7 @@
         <v>dcaf</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>101</v>
       </c>
@@ -2364,7 +2436,7 @@
         <v>daniel</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>103</v>
       </c>
@@ -2379,7 +2451,7 @@
         <v>sofia</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
         <v>66</v>
       </c>
@@ -2393,7 +2465,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
         <v>55</v>
       </c>
@@ -2407,7 +2479,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>58</v>
       </c>
@@ -2421,7 +2493,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>60</v>
       </c>
@@ -2435,7 +2507,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>62</v>
       </c>
@@ -2449,7 +2521,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="8" t="s">
         <v>108</v>
       </c>
@@ -2463,7 +2535,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="8" t="s">
         <v>109</v>
       </c>
@@ -2477,7 +2549,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="36" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>64</v>
       </c>
@@ -2491,7 +2563,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="36" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" ht="36" x14ac:dyDescent="0.3">
       <c r="A41" s="8" t="s">
         <v>112</v>
       </c>
@@ -2505,7 +2577,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="8" t="s">
         <v>114</v>
       </c>
@@ -2519,7 +2591,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="14" t="s">
         <v>126</v>
       </c>
@@ -2527,7 +2599,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="14" t="s">
         <v>127</v>
       </c>
@@ -2535,7 +2607,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
         <v>128</v>
       </c>
@@ -2543,7 +2615,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" s="14" t="s">
         <v>129</v>
       </c>
@@ -2551,7 +2623,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="14" t="s">
         <v>130</v>
       </c>
@@ -2559,7 +2631,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="14" t="s">
         <v>132</v>
       </c>
@@ -2567,7 +2639,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="14" t="s">
         <v>133</v>
       </c>
@@ -2575,7 +2647,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="14" t="s">
         <v>134</v>
       </c>
@@ -2589,6 +2661,34 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <MediaLengthInSeconds xmlns="6f4338ef-addb-4c87-aefe-1895241b335f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08D58FADB61F04EBBB4F355C06EFBED" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="b1e0f6055e0e9a4b9e75d6c71ee7de91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6f4338ef-addb-4c87-aefe-1895241b335f" xmlns:ns3="b91e7f20-fe0a-487d-91a9-605ac1c64acf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b43930f3490e4d4da1ab3f8da7df6f51" ns2:_="" ns3:_="">
     <xsd:import namespace="6f4338ef-addb-4c87-aefe-1895241b335f"/>
@@ -2849,36 +2949,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <MediaLengthInSeconds xmlns="6f4338ef-addb-4c87-aefe-1895241b335f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56D796CB-5E6F-4C55-B925-B0E9D39BDEA9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FCAB9D5-4699-48C8-8DB7-84FDCD7CDA0C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2890,12 +2969,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FCAB9D5-4699-48C8-8DB7-84FDCD7CDA0C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56D796CB-5E6F-4C55-B925-B0E9D39BDEA9}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
-    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>